<commit_message>
Fix link in planning documents & upload them to sprint 2
Signed-off-by: Carl Mosler <carl.mosler@tu-berlin.de>
</commit_message>
<xml_diff>
--- a/Deliverables/sprint-02/planning-documents.xlsx
+++ b/Deliverables/sprint-02/planning-documents.xlsx
@@ -2970,6 +2970,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="12.75"/>
   <cols>
@@ -3185,6 +3186,9 @@
       <c r="D20" s="12"/>
     </row>
   </sheetData>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
   <drawing r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>

</xml_diff>